<commit_message>
tracking update 28.04.2026 11:11
</commit_message>
<xml_diff>
--- a/files/UAE_005_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_25.04.2026.xlsx
+++ b/files/UAE_005_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_25.04.2026.xlsx
@@ -5,17 +5,18 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\UAE\UAE#5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{124B3649-7B08-422E-A6C5-38E62A51E79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6F63D47-EC73-4ACE-9C16-188CCF52835E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э5" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="51">
   <si>
     <t xml:space="preserve">
 Артикул</t>
@@ -181,6 +182,15 @@
   </si>
   <si>
     <t>MERCEDES-BENZ Genuine MB 229.5 5W-40</t>
+  </si>
+  <si>
+    <t>Количество</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Адрес доставки: </t>
+  </si>
+  <si>
+    <t>143930, МО, Балашиха, шоссе Ильича, д. 1</t>
   </si>
 </sst>
 </file>
@@ -6849,7 +6859,7 @@
         <v>0.29593516157289729</v>
       </c>
     </row>
-    <row r="15" spans="1:1022" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1022" ht="15.75" x14ac:dyDescent="0.25">
       <c r="L15" s="6"/>
       <c r="M15" s="6"/>
       <c r="P15" s="44">
@@ -7045,4 +7055,182 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Страница &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{775D4C04-4F24-4937-9FC6-E55E6757B71B}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="59.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>12096</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>5184</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>